<commit_message>
Re-run trial balance report
</commit_message>
<xml_diff>
--- a/input/zostava.xlsx
+++ b/input/zostava.xlsx
@@ -539,16 +539,16 @@
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>962.89</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>962.89</v>
       </c>
       <c r="S6" t="n">
-        <v>-25543.38</v>
+        <v>-26506.27</v>
       </c>
       <c r="T6" t="n">
         <v>0</v>
@@ -699,16 +699,16 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>176.28</v>
       </c>
       <c r="Q8" t="n">
         <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>176.28</v>
       </c>
       <c r="S8" t="n">
-        <v>-333292.37</v>
+        <v>-333468.65</v>
       </c>
       <c r="T8" t="n">
         <v>0</v>
@@ -939,16 +939,16 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>0</v>
+        <v>119.37</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>119.37</v>
       </c>
       <c r="S11" t="n">
-        <v>119.37</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
         <v>0</v>
@@ -975,7 +975,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>191</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -985,12 +985,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Materiál na ceste</t>
+          <t>Opravná položka k materiálu</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1055,7 +1055,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>221</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1065,12 +1065,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Oberbank 2301307910/8370-Kontokerrent</t>
+          <t>Oberbank 2301307910/8370</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1083,32 +1083,26 @@
           <t>2</t>
         </is>
       </c>
-      <c r="K13" t="n">
-        <v>27684.84</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
       <c r="M13" t="n">
-        <v>-27684.84</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>49038.16</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>49038.16</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>49038.16</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>49038.16</v>
       </c>
       <c r="S13" t="n">
-        <v>-27684.84</v>
+        <v>0</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1135,22 +1129,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>231</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Odberatelia - koncern</t>
+          <t>Oberbank 2301307910/8370-Kontokerrent</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1160,35 +1154,35 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>241021.85</v>
-      </c>
-      <c r="J14" t="n">
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>27684.84</v>
+      </c>
+      <c r="L14" t="n">
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>241021.85</v>
+        <v>-27684.84</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>78867.97</v>
+        <v>18745.32</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>78867.97</v>
+        <v>18745.32</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>319889.82</v>
+        <v>-8939.52</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1215,17 +1209,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>261</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>001</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Krátkodobé poskytnuté zálohy</t>
+          <t>Peniaze na ceste</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1240,35 +1234,29 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>9900</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
+          <t>2</t>
+        </is>
       </c>
       <c r="M15" t="n">
-        <v>9900</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="S15" t="n">
-        <v>9900</v>
+        <v>0</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1295,17 +1283,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>315</t>
+          <t>311</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Ostatné pohladávky</t>
+          <t>Odberatelia - koncern</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1324,31 +1312,31 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>554.68</v>
+        <v>241021.85</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>554.68</v>
+        <v>241021.85</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>78867.97</v>
       </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>46635.54</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>78867.97</v>
       </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>46635.54</v>
       </c>
       <c r="S16" t="n">
-        <v>554.68</v>
+        <v>273254.28</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1375,22 +1363,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>314</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>300</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dodávatelia - tuzemsko</t>
+          <t>Krátkodobé poskytnuté zálohy</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1403,14 +1391,14 @@
           <t>3</t>
         </is>
       </c>
-      <c r="K17" t="n">
-        <v>3692.74</v>
-      </c>
-      <c r="L17" t="n">
+      <c r="I17" t="n">
+        <v>9900</v>
+      </c>
+      <c r="J17" t="n">
         <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>-3692.74</v>
+        <v>9900</v>
       </c>
       <c r="N17" t="n">
         <v>0</v>
@@ -1419,16 +1407,16 @@
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>13337.86</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>13337.86</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>-17030.6</v>
+        <v>9900</v>
       </c>
       <c r="T17" t="n">
         <v>0</v>
@@ -1455,22 +1443,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>315</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dodávatelia - koncern</t>
+          <t>Ostatné pohladávky</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1483,14 +1471,14 @@
           <t>3</t>
         </is>
       </c>
-      <c r="K18" t="n">
-        <v>616839.97</v>
-      </c>
-      <c r="L18" t="n">
+      <c r="I18" t="n">
+        <v>554.68</v>
+      </c>
+      <c r="J18" t="n">
         <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>-616839.97</v>
+        <v>554.68</v>
       </c>
       <c r="N18" t="n">
         <v>0</v>
@@ -1499,16 +1487,16 @@
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>4651.39</v>
+        <v>457.68</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>4651.39</v>
+        <v>457.68</v>
       </c>
       <c r="S18" t="n">
-        <v>-621491.36</v>
+        <v>97</v>
       </c>
       <c r="T18" t="n">
         <v>0</v>
@@ -1535,7 +1523,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>321</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1545,7 +1533,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Krátkodobé rezervy nedaňové</t>
+          <t>Dodávatelia - tuzemsko</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1564,31 +1552,31 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>8324.9</v>
+        <v>3692.74</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>-8324.9</v>
+        <v>-3692.74</v>
       </c>
       <c r="N19" t="n">
         <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>4747.38</v>
+        <v>3692.74</v>
       </c>
       <c r="P19" t="n">
-        <v>0</v>
+        <v>13214.86</v>
       </c>
       <c r="Q19" t="n">
-        <v>4747.38</v>
+        <v>3692.74</v>
       </c>
       <c r="R19" t="n">
-        <v>0</v>
+        <v>13214.86</v>
       </c>
       <c r="S19" t="n">
-        <v>-3577.52</v>
+        <v>-13214.86</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1615,17 +1603,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>321</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Krátkodobé rezervy daňové</t>
+          <t>Dodávatelia - koncern</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1644,13 +1632,13 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>12320.53</v>
+        <v>616839.97</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>-12320.53</v>
+        <v>-616839.97</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1659,16 +1647,16 @@
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>0</v>
+        <v>4651.39</v>
       </c>
       <c r="Q20" t="n">
         <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>0</v>
+        <v>4651.39</v>
       </c>
       <c r="S20" t="n">
-        <v>-12320.53</v>
+        <v>-621491.36</v>
       </c>
       <c r="T20" t="n">
         <v>0</v>
@@ -1695,17 +1683,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>325</t>
+          <t>323</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>001</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ostatné zaväzky-nájom</t>
+          <t>Krátkodobé rezervy nedaňové</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1723,26 +1711,32 @@
           <t>3</t>
         </is>
       </c>
+      <c r="K21" t="n">
+        <v>8324.9</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>-8324.9</v>
       </c>
       <c r="N21" t="n">
         <v>0</v>
       </c>
       <c r="O21" t="n">
-        <v>0</v>
+        <v>4647.38</v>
       </c>
       <c r="P21" t="n">
-        <v>6951.75</v>
+        <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>4647.38</v>
       </c>
       <c r="R21" t="n">
-        <v>6951.75</v>
+        <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>-6951.75</v>
+        <v>-3677.52</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1769,17 +1763,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>331</t>
+          <t>323</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Zamestnanci</t>
+          <t>Krátkodobé rezervy daňové</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1797,14 +1791,14 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I22" t="n">
-        <v>-15134.28</v>
-      </c>
-      <c r="J22" t="n">
+      <c r="K22" t="n">
+        <v>12320.53</v>
+      </c>
+      <c r="L22" t="n">
         <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>-15134.28</v>
+        <v>-12320.53</v>
       </c>
       <c r="N22" t="n">
         <v>0</v>
@@ -1822,7 +1816,7 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>-15134.28</v>
+        <v>-12320.53</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -1849,17 +1843,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>325</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Ost.záväzky voci zamestnancom</t>
+          <t>Ostatné zaväzky-nájom</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1877,14 +1871,8 @@
           <t>3</t>
         </is>
       </c>
-      <c r="K23" t="n">
-        <v>180</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
       <c r="M23" t="n">
-        <v>-180</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
         <v>0</v>
@@ -1893,16 +1881,16 @@
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>0</v>
+        <v>6951.75</v>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
       </c>
       <c r="R23" t="n">
-        <v>0</v>
+        <v>6951.75</v>
       </c>
       <c r="S23" t="n">
-        <v>-180</v>
+        <v>-6951.75</v>
       </c>
       <c r="T23" t="n">
         <v>0</v>
@@ -1929,22 +1917,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>335</t>
+          <t>331</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>001</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pohĺ.voči zam-com-pokladna-EUR</t>
+          <t>Zamestnanci</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1958,31 +1946,31 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>188.79</v>
+        <v>-15134.28</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>188.79</v>
+        <v>-15134.28</v>
       </c>
       <c r="N24" t="n">
         <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>19878.77</v>
       </c>
       <c r="P24" t="n">
-        <v>0</v>
+        <v>20800.79</v>
       </c>
       <c r="Q24" t="n">
-        <v>0</v>
+        <v>19878.77</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>20800.79</v>
       </c>
       <c r="S24" t="n">
-        <v>188.79</v>
+        <v>-16056.3</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2009,17 +1997,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>336</t>
+          <t>333</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Zdravotné poistenie</t>
+          <t>Ost.záväzky voci zamestnancom</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2038,31 +2026,31 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>2836.62</v>
+        <v>180</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>-2836.62</v>
+        <v>-180</v>
       </c>
       <c r="N25" t="n">
         <v>0</v>
       </c>
       <c r="O25" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>-2836.62</v>
+        <v>0</v>
       </c>
       <c r="T25" t="n">
         <v>0</v>
@@ -2089,22 +2077,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>336</t>
+          <t>335</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Sociálne poistenie</t>
+          <t>Pohĺad. voči zamestn.-obedy</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2117,32 +2105,26 @@
           <t>3</t>
         </is>
       </c>
-      <c r="K26" t="n">
-        <v>6542.45</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
       <c r="M26" t="n">
-        <v>-6542.45</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
+        <v>271.8</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>271.8</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>271.8</v>
       </c>
       <c r="R26" t="n">
-        <v>0</v>
+        <v>271.8</v>
       </c>
       <c r="S26" t="n">
-        <v>-6542.45</v>
+        <v>0</v>
       </c>
       <c r="T26" t="n">
         <v>0</v>
@@ -2169,22 +2151,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>335</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>400</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Daň z príjmov</t>
+          <t>Pohĺ.voči zam-com-pokladna-EUR</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2197,32 +2179,32 @@
           <t>3</t>
         </is>
       </c>
-      <c r="K27" t="n">
-        <v>3840</v>
-      </c>
-      <c r="L27" t="n">
+      <c r="I27" t="n">
+        <v>188.79</v>
+      </c>
+      <c r="J27" t="n">
         <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>-3840</v>
+        <v>188.79</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="P27" t="n">
-        <v>0</v>
+        <v>132.85</v>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="R27" t="n">
-        <v>0</v>
+        <v>132.85</v>
       </c>
       <c r="S27" t="n">
-        <v>-3840</v>
+        <v>455.94</v>
       </c>
       <c r="T27" t="n">
         <v>0</v>
@@ -2249,17 +2231,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>342</t>
+          <t>336</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ostatné priame dane</t>
+          <t>Zdravotné poistenie</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2278,31 +2260,31 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>963.14</v>
+        <v>2836.62</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>-963.14</v>
+        <v>-2836.62</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>0</v>
+        <v>2836.62</v>
       </c>
       <c r="P28" t="n">
-        <v>0</v>
+        <v>3171.53</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>2836.62</v>
       </c>
       <c r="R28" t="n">
-        <v>0</v>
+        <v>3171.53</v>
       </c>
       <c r="S28" t="n">
-        <v>-963.14</v>
+        <v>-3171.53</v>
       </c>
       <c r="T28" t="n">
         <v>0</v>
@@ -2329,17 +2311,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>343</t>
+          <t>336</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>RCH výstup</t>
+          <t>Sociálne poistenie</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2357,26 +2339,32 @@
           <t>3</t>
         </is>
       </c>
+      <c r="K29" t="n">
+        <v>6542.45</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>-6542.45</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>0</v>
+        <v>6542.45</v>
       </c>
       <c r="P29" t="n">
-        <v>1069.82</v>
+        <v>6857.88</v>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
+        <v>6542.45</v>
       </c>
       <c r="R29" t="n">
-        <v>1069.82</v>
+        <v>6857.88</v>
       </c>
       <c r="S29" t="n">
-        <v>-1069.82</v>
+        <v>-6857.88</v>
       </c>
       <c r="T29" t="n">
         <v>0</v>
@@ -2403,17 +2391,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>343</t>
+          <t>341</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DPH na vstupe</t>
+          <t>Daň z príjmov</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2431,26 +2419,32 @@
           <t>3</t>
         </is>
       </c>
+      <c r="K30" t="n">
+        <v>3840</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>-3840</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>3676.3</v>
+        <v>0</v>
       </c>
       <c r="P30" t="n">
         <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>3676.3</v>
+        <v>0</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>3676.3</v>
+        <v>-3840</v>
       </c>
       <c r="T30" t="n">
         <v>0</v>
@@ -2477,17 +2471,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>343</t>
+          <t>342</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>001</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>RCH vstup</t>
+          <t>Ostatné priame dane</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2505,26 +2499,32 @@
           <t>3</t>
         </is>
       </c>
+      <c r="K31" t="n">
+        <v>963.14</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>-963.14</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>
       </c>
       <c r="O31" t="n">
-        <v>1069.82</v>
+        <v>1563.14</v>
       </c>
       <c r="P31" t="n">
-        <v>0</v>
+        <v>1618.58</v>
       </c>
       <c r="Q31" t="n">
-        <v>1069.82</v>
+        <v>1563.14</v>
       </c>
       <c r="R31" t="n">
-        <v>0</v>
+        <v>1618.58</v>
       </c>
       <c r="S31" t="n">
-        <v>1069.82</v>
+        <v>-1018.58</v>
       </c>
       <c r="T31" t="n">
         <v>0</v>
@@ -2556,12 +2556,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DPH Voči daňovému úradu</t>
+          <t>DPH na vystupe</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2579,14 +2579,8 @@
           <t>3</t>
         </is>
       </c>
-      <c r="K32" t="n">
-        <v>-9694.27</v>
-      </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
       <c r="M32" t="n">
-        <v>9694.27</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
         <v>0</v>
@@ -2595,16 +2589,16 @@
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>0</v>
+        <v>43.4</v>
       </c>
       <c r="Q32" t="n">
         <v>0</v>
       </c>
       <c r="R32" t="n">
-        <v>0</v>
+        <v>43.4</v>
       </c>
       <c r="S32" t="n">
-        <v>9694.27</v>
+        <v>-43.4</v>
       </c>
       <c r="T32" t="n">
         <v>0</v>
@@ -2631,17 +2625,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>345</t>
+          <t>343</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ostatné dane a poplatky</t>
+          <t>RCH výstup</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2659,14 +2653,8 @@
           <t>3</t>
         </is>
       </c>
-      <c r="K33" t="n">
-        <v>323.83</v>
-      </c>
-      <c r="L33" t="n">
-        <v>0</v>
-      </c>
       <c r="M33" t="n">
-        <v>-323.83</v>
+        <v>0</v>
       </c>
       <c r="N33" t="n">
         <v>0</v>
@@ -2675,16 +2663,16 @@
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>0</v>
+        <v>1069.82</v>
       </c>
       <c r="Q33" t="n">
         <v>0</v>
       </c>
       <c r="R33" t="n">
-        <v>0</v>
+        <v>1069.82</v>
       </c>
       <c r="S33" t="n">
-        <v>-323.83</v>
+        <v>-1069.82</v>
       </c>
       <c r="T33" t="n">
         <v>0</v>
@@ -2711,17 +2699,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>379</t>
+          <t>343</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>400</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ostatné záväzky</t>
+          <t>DPH na vstupe</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2746,19 +2734,19 @@
         <v>0</v>
       </c>
       <c r="O34" t="n">
-        <v>0</v>
+        <v>3671.04</v>
       </c>
       <c r="P34" t="n">
-        <v>1158.84</v>
+        <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>0</v>
+        <v>3671.04</v>
       </c>
       <c r="R34" t="n">
-        <v>1158.84</v>
+        <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>-1158.84</v>
+        <v>3671.04</v>
       </c>
       <c r="T34" t="n">
         <v>0</v>
@@ -2785,22 +2773,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>343</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>410</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Náklady budúcich období-ostatné</t>
+          <t>RCH vstup</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2813,32 +2801,26 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I35" t="n">
-        <v>300.69</v>
-      </c>
-      <c r="J35" t="n">
-        <v>0</v>
-      </c>
       <c r="M35" t="n">
-        <v>300.69</v>
+        <v>0</v>
       </c>
       <c r="N35" t="n">
         <v>0</v>
       </c>
       <c r="O35" t="n">
-        <v>0</v>
+        <v>1069.82</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>0</v>
+        <v>1069.82</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>300.69</v>
+        <v>1069.82</v>
       </c>
       <c r="T35" t="n">
         <v>0</v>
@@ -2865,22 +2847,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>343</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>900</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Nákl.bud.obd.ostatné-dlhod.</t>
+          <t>DPH Voči daňovému úradu</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2893,14 +2875,14 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I36" t="n">
-        <v>8.01</v>
-      </c>
-      <c r="J36" t="n">
+      <c r="K36" t="n">
+        <v>-9694.27</v>
+      </c>
+      <c r="L36" t="n">
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>8.01</v>
+        <v>9694.27</v>
       </c>
       <c r="N36" t="n">
         <v>0</v>
@@ -2909,16 +2891,16 @@
         <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>1944.94</v>
       </c>
       <c r="Q36" t="n">
         <v>0</v>
       </c>
       <c r="R36" t="n">
-        <v>0</v>
+        <v>1944.94</v>
       </c>
       <c r="S36" t="n">
-        <v>8.01</v>
+        <v>7749.33</v>
       </c>
       <c r="T36" t="n">
         <v>0</v>
@@ -2945,17 +2927,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>383</t>
+          <t>345</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Vydavky budúcich období</t>
+          <t>Ostatné dane a poplatky</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2974,31 +2956,31 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>0.78</v>
+        <v>323.83</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>-0.78</v>
+        <v>-323.83</v>
       </c>
       <c r="N37" t="n">
         <v>0</v>
       </c>
       <c r="O37" t="n">
-        <v>0</v>
+        <v>323.83</v>
       </c>
       <c r="P37" t="n">
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
+        <v>323.83</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>-0.78</v>
+        <v>0</v>
       </c>
       <c r="T37" t="n">
         <v>0</v>
@@ -3025,17 +3007,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>379</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>900</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Základné imanie</t>
+          <t>Ostatné záväzky</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3050,17 +3032,11 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="K38" t="n">
-        <v>6639</v>
-      </c>
-      <c r="L38" t="n">
-        <v>0</v>
+          <t>3</t>
+        </is>
       </c>
       <c r="M38" t="n">
-        <v>-6639</v>
+        <v>0</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
@@ -3069,16 +3045,16 @@
         <v>0</v>
       </c>
       <c r="P38" t="n">
-        <v>0</v>
+        <v>1158.84</v>
       </c>
       <c r="Q38" t="n">
         <v>0</v>
       </c>
       <c r="R38" t="n">
-        <v>0</v>
+        <v>1158.84</v>
       </c>
       <c r="S38" t="n">
-        <v>-6639</v>
+        <v>-1158.84</v>
       </c>
       <c r="T38" t="n">
         <v>0</v>
@@ -3105,22 +3081,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>413</t>
+          <t>381</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Ostatné kapitálové fondy</t>
+          <t>Náklady budúcich období-ostatné</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3130,17 +3106,17 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="K39" t="n">
-        <v>100000</v>
-      </c>
-      <c r="L39" t="n">
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>300.69</v>
+      </c>
+      <c r="J39" t="n">
         <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>-100000</v>
+        <v>300.69</v>
       </c>
       <c r="N39" t="n">
         <v>0</v>
@@ -3158,7 +3134,7 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>-100000</v>
+        <v>300.69</v>
       </c>
       <c r="T39" t="n">
         <v>0</v>
@@ -3185,22 +3161,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>421</t>
+          <t>381</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>300</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Zakonný rezervný fond</t>
+          <t>Nákl.bud.obd.ostatné-dlhod.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3210,17 +3186,17 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="K40" t="n">
-        <v>663.88</v>
-      </c>
-      <c r="L40" t="n">
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>8.01</v>
+      </c>
+      <c r="J40" t="n">
         <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>-663.88</v>
+        <v>8.01</v>
       </c>
       <c r="N40" t="n">
         <v>0</v>
@@ -3238,7 +3214,7 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>-663.88</v>
+        <v>8.01</v>
       </c>
       <c r="T40" t="n">
         <v>0</v>
@@ -3265,7 +3241,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>429</t>
+          <t>383</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3275,7 +3251,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Neuhradená strata min. rokov</t>
+          <t>Vydavky budúcich období</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3290,17 +3266,17 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="K41" t="n">
-        <v>-59798.94</v>
+        <v>0.78</v>
       </c>
       <c r="L41" t="n">
         <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>59798.94</v>
+        <v>-0.78</v>
       </c>
       <c r="N41" t="n">
         <v>0</v>
@@ -3318,7 +3294,7 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>59798.94</v>
+        <v>-0.78</v>
       </c>
       <c r="T41" t="n">
         <v>0</v>
@@ -3345,7 +3321,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>411</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3355,7 +3331,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Výsledok hospodárenia v schv.</t>
+          <t>Základné imanie</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3373,14 +3349,14 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I42" t="n">
-        <v>295302.52</v>
-      </c>
-      <c r="J42" t="n">
+      <c r="K42" t="n">
+        <v>6639</v>
+      </c>
+      <c r="L42" t="n">
         <v>0</v>
       </c>
       <c r="M42" t="n">
-        <v>295302.52</v>
+        <v>-6639</v>
       </c>
       <c r="N42" t="n">
         <v>0</v>
@@ -3398,7 +3374,7 @@
         <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>295302.52</v>
+        <v>-6639</v>
       </c>
       <c r="T42" t="n">
         <v>0</v>
@@ -3425,7 +3401,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>413</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3435,7 +3411,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Ostatné rezervy</t>
+          <t>Ostatné kapitálové fondy</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3454,13 +3430,13 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>3038.99</v>
+        <v>100000</v>
       </c>
       <c r="L43" t="n">
         <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>-3038.99</v>
+        <v>-100000</v>
       </c>
       <c r="N43" t="n">
         <v>0</v>
@@ -3478,7 +3454,7 @@
         <v>0</v>
       </c>
       <c r="S43" t="n">
-        <v>-3038.99</v>
+        <v>-100000</v>
       </c>
       <c r="T43" t="n">
         <v>0</v>
@@ -3505,7 +3481,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>472</t>
+          <t>421</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3515,7 +3491,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Záväzky zo sociálneho fondu</t>
+          <t>Zakonný rezervný fond</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3534,13 +3510,13 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>9480.69</v>
+        <v>663.88</v>
       </c>
       <c r="L44" t="n">
         <v>0</v>
       </c>
       <c r="M44" t="n">
-        <v>-9480.69</v>
+        <v>-663.88</v>
       </c>
       <c r="N44" t="n">
         <v>0</v>
@@ -3558,7 +3534,7 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>-9480.69</v>
+        <v>-663.88</v>
       </c>
       <c r="T44" t="n">
         <v>0</v>
@@ -3585,17 +3561,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>479</t>
+          <t>429</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Slovak Telecom-krátkodobá časť</t>
+          <t>Neuhradená strata min. rokov</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3614,31 +3590,31 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>19</v>
+        <v>-59798.94</v>
       </c>
       <c r="L45" t="n">
         <v>0</v>
       </c>
       <c r="M45" t="n">
-        <v>-19</v>
+        <v>59798.94</v>
       </c>
       <c r="N45" t="n">
         <v>0</v>
       </c>
       <c r="O45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
         <v>0</v>
       </c>
       <c r="Q45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R45" t="n">
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>-17</v>
+        <v>59798.94</v>
       </c>
       <c r="T45" t="n">
         <v>0</v>
@@ -3665,17 +3641,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>479</t>
+          <t>431</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Tatra Leasing-krátkodobá časť spot.úver</t>
+          <t>Výsledok hospodárenia v schv.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3693,32 +3669,32 @@
           <t>4</t>
         </is>
       </c>
-      <c r="K46" t="n">
-        <v>9940.06</v>
-      </c>
-      <c r="L46" t="n">
+      <c r="I46" t="n">
+        <v>295302.52</v>
+      </c>
+      <c r="J46" t="n">
         <v>0</v>
       </c>
       <c r="M46" t="n">
-        <v>-9940.06</v>
+        <v>295302.52</v>
       </c>
       <c r="N46" t="n">
         <v>0</v>
       </c>
       <c r="O46" t="n">
-        <v>810.5</v>
+        <v>0</v>
       </c>
       <c r="P46" t="n">
         <v>0</v>
       </c>
       <c r="Q46" t="n">
-        <v>810.5</v>
+        <v>0</v>
       </c>
       <c r="R46" t="n">
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>-9129.56</v>
+        <v>295302.52</v>
       </c>
       <c r="T46" t="n">
         <v>0</v>
@@ -3745,17 +3721,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>479</t>
+          <t>459</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Tatra Leasing-dlhodobá časť spot.úver</t>
+          <t>Ostatné rezervy</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3774,13 +3750,13 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>28924.78</v>
+        <v>3038.99</v>
       </c>
       <c r="L47" t="n">
         <v>0</v>
       </c>
       <c r="M47" t="n">
-        <v>-28924.78</v>
+        <v>-3038.99</v>
       </c>
       <c r="N47" t="n">
         <v>0</v>
@@ -3798,7 +3774,7 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>-28924.78</v>
+        <v>-3038.99</v>
       </c>
       <c r="T47" t="n">
         <v>0</v>
@@ -3825,22 +3801,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>501</t>
+          <t>472</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Spotr.mat.prevádzka</t>
+          <t>Záväzky zo sociálneho fondu</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3850,29 +3826,35 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>9480.69</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0</v>
       </c>
       <c r="M48" t="n">
-        <v>0</v>
+        <v>-9480.69</v>
       </c>
       <c r="N48" t="n">
         <v>0</v>
       </c>
       <c r="O48" t="n">
-        <v>123</v>
+        <v>0</v>
       </c>
       <c r="P48" t="n">
         <v>0</v>
       </c>
       <c r="Q48" t="n">
-        <v>123</v>
+        <v>0</v>
       </c>
       <c r="R48" t="n">
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>123</v>
+        <v>-9480.69</v>
       </c>
       <c r="T48" t="n">
         <v>0</v>
@@ -3899,22 +3881,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>501</t>
+          <t>479</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PHM AA944RK</t>
+          <t>Slovak Telecom-krátkodobá časť</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3924,29 +3906,35 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>19</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0</v>
       </c>
       <c r="M49" t="n">
-        <v>0</v>
+        <v>-19</v>
       </c>
       <c r="N49" t="n">
         <v>0</v>
       </c>
       <c r="O49" t="n">
-        <v>101.62</v>
+        <v>2</v>
       </c>
       <c r="P49" t="n">
         <v>0</v>
       </c>
       <c r="Q49" t="n">
-        <v>101.62</v>
+        <v>2</v>
       </c>
       <c r="R49" t="n">
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>101.62</v>
+        <v>-17</v>
       </c>
       <c r="T49" t="n">
         <v>0</v>
@@ -3973,22 +3961,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>501</t>
+          <t>479</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>400</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PHM NR600LP</t>
+          <t>Tatra Leasing-krátkodobá časť spot.úver</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3998,29 +3986,35 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>9940.06</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0</v>
       </c>
       <c r="M50" t="n">
-        <v>0</v>
+        <v>-9940.06</v>
       </c>
       <c r="N50" t="n">
         <v>0</v>
       </c>
       <c r="O50" t="n">
-        <v>23.48</v>
+        <v>810.5</v>
       </c>
       <c r="P50" t="n">
         <v>0</v>
       </c>
       <c r="Q50" t="n">
-        <v>23.48</v>
+        <v>810.5</v>
       </c>
       <c r="R50" t="n">
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>23.48</v>
+        <v>-9129.56</v>
       </c>
       <c r="T50" t="n">
         <v>0</v>
@@ -4047,22 +4041,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>501</t>
+          <t>479</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>500</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Amadys-Spotr.mat.výr.</t>
+          <t>Tatra Leasing-dlhodobá časť spot.úver</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4072,29 +4066,35 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>28924.78</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0</v>
       </c>
       <c r="M51" t="n">
-        <v>0</v>
+        <v>-28924.78</v>
       </c>
       <c r="N51" t="n">
         <v>0</v>
       </c>
       <c r="O51" t="n">
-        <v>4651.39</v>
+        <v>0</v>
       </c>
       <c r="P51" t="n">
         <v>0</v>
       </c>
       <c r="Q51" t="n">
-        <v>4651.39</v>
+        <v>0</v>
       </c>
       <c r="R51" t="n">
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>4651.39</v>
+        <v>-28924.78</v>
       </c>
       <c r="T51" t="n">
         <v>0</v>
@@ -4126,12 +4126,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>990</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>spotreba PHM-nedanová</t>
+          <t>Kancelárske potreby</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -4156,19 +4156,19 @@
         <v>0</v>
       </c>
       <c r="O52" t="n">
-        <v>153.85</v>
+        <v>22.28</v>
       </c>
       <c r="P52" t="n">
         <v>0</v>
       </c>
       <c r="Q52" t="n">
-        <v>153.85</v>
+        <v>22.28</v>
       </c>
       <c r="R52" t="n">
         <v>0</v>
       </c>
       <c r="S52" t="n">
-        <v>153.85</v>
+        <v>22.28</v>
       </c>
       <c r="T52" t="n">
         <v>0</v>
@@ -4195,17 +4195,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>502</t>
+          <t>501</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>300</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Spotreba el. energie</t>
+          <t>Spotreba obalového materiálu</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4230,19 +4230,19 @@
         <v>0</v>
       </c>
       <c r="O53" t="n">
-        <v>506.25</v>
+        <v>28.86</v>
       </c>
       <c r="P53" t="n">
         <v>0</v>
       </c>
       <c r="Q53" t="n">
-        <v>506.25</v>
+        <v>28.86</v>
       </c>
       <c r="R53" t="n">
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>506.25</v>
+        <v>28.86</v>
       </c>
       <c r="T53" t="n">
         <v>0</v>
@@ -4269,17 +4269,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>502</t>
+          <t>501</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>360</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Spotreba ostatnej energie</t>
+          <t>Spotr.mat.prevádzka</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -4304,19 +4304,19 @@
         <v>0</v>
       </c>
       <c r="O54" t="n">
-        <v>306.25</v>
+        <v>144.09</v>
       </c>
       <c r="P54" t="n">
         <v>0</v>
       </c>
       <c r="Q54" t="n">
-        <v>306.25</v>
+        <v>144.09</v>
       </c>
       <c r="R54" t="n">
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>306.25</v>
+        <v>144.09</v>
       </c>
       <c r="T54" t="n">
         <v>0</v>
@@ -4343,17 +4343,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>513</t>
+          <t>501</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>450</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Náklady na reprezentáciu</t>
+          <t>PHM AA944RK</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -4378,19 +4378,19 @@
         <v>0</v>
       </c>
       <c r="O55" t="n">
-        <v>150.95</v>
+        <v>159.02</v>
       </c>
       <c r="P55" t="n">
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>150.95</v>
+        <v>159.02</v>
       </c>
       <c r="R55" t="n">
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>150.95</v>
+        <v>159.02</v>
       </c>
       <c r="T55" t="n">
         <v>0</v>
@@ -4417,17 +4417,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>518</t>
+          <t>501</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>460</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Telefon, internet</t>
+          <t>PHM NR600LP</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -4452,19 +4452,19 @@
         <v>0</v>
       </c>
       <c r="O56" t="n">
-        <v>115.61</v>
+        <v>85.45</v>
       </c>
       <c r="P56" t="n">
         <v>0</v>
       </c>
       <c r="Q56" t="n">
-        <v>115.61</v>
+        <v>85.45</v>
       </c>
       <c r="R56" t="n">
         <v>0</v>
       </c>
       <c r="S56" t="n">
-        <v>115.61</v>
+        <v>85.45</v>
       </c>
       <c r="T56" t="n">
         <v>0</v>
@@ -4491,17 +4491,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>518</t>
+          <t>501</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>600</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Nájomné</t>
+          <t>Amadys-Spotr.mat.výr.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -4526,19 +4526,19 @@
         <v>0</v>
       </c>
       <c r="O57" t="n">
-        <v>4108.33</v>
+        <v>4651.39</v>
       </c>
       <c r="P57" t="n">
         <v>0</v>
       </c>
       <c r="Q57" t="n">
-        <v>4108.33</v>
+        <v>4651.39</v>
       </c>
       <c r="R57" t="n">
         <v>0</v>
       </c>
       <c r="S57" t="n">
-        <v>4108.33</v>
+        <v>4651.39</v>
       </c>
       <c r="T57" t="n">
         <v>0</v>
@@ -4565,17 +4565,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>518</t>
+          <t>501</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>990</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Služby spojené s nájmom</t>
+          <t>spotreba PHM-nedanová</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -4600,19 +4600,19 @@
         <v>0</v>
       </c>
       <c r="O58" t="n">
-        <v>1350</v>
+        <v>153.85</v>
       </c>
       <c r="P58" t="n">
         <v>0</v>
       </c>
       <c r="Q58" t="n">
-        <v>1350</v>
+        <v>153.85</v>
       </c>
       <c r="R58" t="n">
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>1350</v>
+        <v>153.85</v>
       </c>
       <c r="T58" t="n">
         <v>0</v>
@@ -4639,17 +4639,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>518</t>
+          <t>502</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Prenájom - ostatné</t>
+          <t>Spotreba el. energie</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4674,19 +4674,19 @@
         <v>0</v>
       </c>
       <c r="O59" t="n">
-        <v>2059</v>
+        <v>506.25</v>
       </c>
       <c r="P59" t="n">
         <v>0</v>
       </c>
       <c r="Q59" t="n">
-        <v>2059</v>
+        <v>506.25</v>
       </c>
       <c r="R59" t="n">
         <v>0</v>
       </c>
       <c r="S59" t="n">
-        <v>2059</v>
+        <v>506.25</v>
       </c>
       <c r="T59" t="n">
         <v>0</v>
@@ -4713,17 +4713,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>518</t>
+          <t>502</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>900</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Služby-ochr.pred požiarmi,BOZP</t>
+          <t>Spotreba ostatnej energie</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4748,19 +4748,19 @@
         <v>0</v>
       </c>
       <c r="O60" t="n">
-        <v>150</v>
+        <v>306.25</v>
       </c>
       <c r="P60" t="n">
         <v>0</v>
       </c>
       <c r="Q60" t="n">
-        <v>150</v>
+        <v>306.25</v>
       </c>
       <c r="R60" t="n">
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>150</v>
+        <v>306.25</v>
       </c>
       <c r="T60" t="n">
         <v>0</v>
@@ -4787,17 +4787,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>518</t>
+          <t>511</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Prepravné, kuriérske služby</t>
+          <t>Opravy a údržba NR 600 LP</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4822,19 +4822,19 @@
         <v>0</v>
       </c>
       <c r="O61" t="n">
-        <v>1960</v>
+        <v>4.88</v>
       </c>
       <c r="P61" t="n">
         <v>0</v>
       </c>
       <c r="Q61" t="n">
-        <v>1960</v>
+        <v>4.88</v>
       </c>
       <c r="R61" t="n">
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>1960</v>
+        <v>4.88</v>
       </c>
       <c r="T61" t="n">
         <v>0</v>
@@ -4861,17 +4861,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>527</t>
+          <t>511</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>990</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Stravovanie zamestnancov</t>
+          <t>Opravy a údržba NR 600 LP nedaňové</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4896,19 +4896,19 @@
         <v>0</v>
       </c>
       <c r="O62" t="n">
-        <v>632.69</v>
+        <v>6</v>
       </c>
       <c r="P62" t="n">
         <v>0</v>
       </c>
       <c r="Q62" t="n">
-        <v>632.69</v>
+        <v>6</v>
       </c>
       <c r="R62" t="n">
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>632.69</v>
+        <v>6</v>
       </c>
       <c r="T62" t="n">
         <v>0</v>
@@ -4935,17 +4935,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>528</t>
+          <t>512</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>130</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Stravovanie nad limit</t>
+          <t>Diéty do limitu</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4970,19 +4970,19 @@
         <v>0</v>
       </c>
       <c r="O63" t="n">
-        <v>122.9</v>
+        <v>180</v>
       </c>
       <c r="P63" t="n">
         <v>0</v>
       </c>
       <c r="Q63" t="n">
-        <v>122.9</v>
+        <v>180</v>
       </c>
       <c r="R63" t="n">
         <v>0</v>
       </c>
       <c r="S63" t="n">
-        <v>122.9</v>
+        <v>180</v>
       </c>
       <c r="T63" t="n">
         <v>0</v>
@@ -5009,17 +5009,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>548</t>
+          <t>513</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Poistenie</t>
+          <t>Náklady na reprezentáciu</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -5044,19 +5044,19 @@
         <v>0</v>
       </c>
       <c r="O64" t="n">
-        <v>194.83</v>
+        <v>182.95</v>
       </c>
       <c r="P64" t="n">
         <v>0</v>
       </c>
       <c r="Q64" t="n">
-        <v>194.83</v>
+        <v>182.95</v>
       </c>
       <c r="R64" t="n">
         <v>0</v>
       </c>
       <c r="S64" t="n">
-        <v>194.83</v>
+        <v>182.95</v>
       </c>
       <c r="T64" t="n">
         <v>0</v>
@@ -5083,7 +5083,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>562</t>
+          <t>518</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Nákladové úroky AA944RK</t>
+          <t>Telefon, internet</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -5118,19 +5118,19 @@
         <v>0</v>
       </c>
       <c r="O65" t="n">
-        <v>153.51</v>
+        <v>115.61</v>
       </c>
       <c r="P65" t="n">
         <v>0</v>
       </c>
       <c r="Q65" t="n">
-        <v>153.51</v>
+        <v>115.61</v>
       </c>
       <c r="R65" t="n">
         <v>0</v>
       </c>
       <c r="S65" t="n">
-        <v>153.51</v>
+        <v>115.61</v>
       </c>
       <c r="T65" t="n">
         <v>0</v>
@@ -5157,74 +5157,1406 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>518</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Nájomné</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0</v>
+      </c>
+      <c r="O66" t="n">
+        <v>4108.33</v>
+      </c>
+      <c r="P66" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>4108.33</v>
+      </c>
+      <c r="R66" t="n">
+        <v>0</v>
+      </c>
+      <c r="S66" t="n">
+        <v>4108.33</v>
+      </c>
+      <c r="T66" t="n">
+        <v>0</v>
+      </c>
+      <c r="U66" t="n">
+        <v>0</v>
+      </c>
+      <c r="V66" t="n">
+        <v>0</v>
+      </c>
+      <c r="W66" t="n">
+        <v>0</v>
+      </c>
+      <c r="X66" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y66" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z66" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Služby spojené s nájmom</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" t="n">
+        <v>1350</v>
+      </c>
+      <c r="P67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>1350</v>
+      </c>
+      <c r="R67" t="n">
+        <v>0</v>
+      </c>
+      <c r="S67" t="n">
+        <v>1350</v>
+      </c>
+      <c r="T67" t="n">
+        <v>0</v>
+      </c>
+      <c r="U67" t="n">
+        <v>0</v>
+      </c>
+      <c r="V67" t="n">
+        <v>0</v>
+      </c>
+      <c r="W67" t="n">
+        <v>0</v>
+      </c>
+      <c r="X67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y67" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z67" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Prenájom - ostatné</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M68" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" t="n">
+        <v>0</v>
+      </c>
+      <c r="O68" t="n">
+        <v>2059</v>
+      </c>
+      <c r="P68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>2059</v>
+      </c>
+      <c r="R68" t="n">
+        <v>0</v>
+      </c>
+      <c r="S68" t="n">
+        <v>2059</v>
+      </c>
+      <c r="T68" t="n">
+        <v>0</v>
+      </c>
+      <c r="U68" t="n">
+        <v>0</v>
+      </c>
+      <c r="V68" t="n">
+        <v>0</v>
+      </c>
+      <c r="W68" t="n">
+        <v>0</v>
+      </c>
+      <c r="X68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y68" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z68" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Služby-ochr.pred požiarmi,BOZP</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M69" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" t="n">
+        <v>150</v>
+      </c>
+      <c r="P69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>150</v>
+      </c>
+      <c r="R69" t="n">
+        <v>0</v>
+      </c>
+      <c r="S69" t="n">
+        <v>150</v>
+      </c>
+      <c r="T69" t="n">
+        <v>0</v>
+      </c>
+      <c r="U69" t="n">
+        <v>0</v>
+      </c>
+      <c r="V69" t="n">
+        <v>0</v>
+      </c>
+      <c r="W69" t="n">
+        <v>0</v>
+      </c>
+      <c r="X69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z69" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Prepravné, kuriérske služby</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M70" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" t="n">
+        <v>0</v>
+      </c>
+      <c r="O70" t="n">
+        <v>1960</v>
+      </c>
+      <c r="P70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>1960</v>
+      </c>
+      <c r="R70" t="n">
+        <v>0</v>
+      </c>
+      <c r="S70" t="n">
+        <v>1960</v>
+      </c>
+      <c r="T70" t="n">
+        <v>0</v>
+      </c>
+      <c r="U70" t="n">
+        <v>0</v>
+      </c>
+      <c r="V70" t="n">
+        <v>0</v>
+      </c>
+      <c r="W70" t="n">
+        <v>0</v>
+      </c>
+      <c r="X70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y70" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z70" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>521</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Mzdové náklady</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" t="n">
+        <v>19823.19</v>
+      </c>
+      <c r="P71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>19823.19</v>
+      </c>
+      <c r="R71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S71" t="n">
+        <v>19823.19</v>
+      </c>
+      <c r="T71" t="n">
+        <v>0</v>
+      </c>
+      <c r="U71" t="n">
+        <v>0</v>
+      </c>
+      <c r="V71" t="n">
+        <v>0</v>
+      </c>
+      <c r="W71" t="n">
+        <v>0</v>
+      </c>
+      <c r="X71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z71" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>524</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Zdravotné poistenie</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M72" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" t="n">
+        <v>2180.46</v>
+      </c>
+      <c r="P72" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>2180.46</v>
+      </c>
+      <c r="R72" t="n">
+        <v>0</v>
+      </c>
+      <c r="S72" t="n">
+        <v>2180.46</v>
+      </c>
+      <c r="T72" t="n">
+        <v>0</v>
+      </c>
+      <c r="U72" t="n">
+        <v>0</v>
+      </c>
+      <c r="V72" t="n">
+        <v>0</v>
+      </c>
+      <c r="W72" t="n">
+        <v>0</v>
+      </c>
+      <c r="X72" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y72" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z72" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>524</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Sociálne poistenie</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M73" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" t="n">
+        <v>4994.84</v>
+      </c>
+      <c r="P73" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>4994.84</v>
+      </c>
+      <c r="R73" t="n">
+        <v>0</v>
+      </c>
+      <c r="S73" t="n">
+        <v>4994.84</v>
+      </c>
+      <c r="T73" t="n">
+        <v>0</v>
+      </c>
+      <c r="U73" t="n">
+        <v>0</v>
+      </c>
+      <c r="V73" t="n">
+        <v>0</v>
+      </c>
+      <c r="W73" t="n">
+        <v>0</v>
+      </c>
+      <c r="X73" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y73" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z73" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>527</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Stravovanie zamestnancov</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M74" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" t="n">
+        <v>632.69</v>
+      </c>
+      <c r="P74" t="n">
+        <v>228.4</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>632.69</v>
+      </c>
+      <c r="R74" t="n">
+        <v>228.4</v>
+      </c>
+      <c r="S74" t="n">
+        <v>404.29</v>
+      </c>
+      <c r="T74" t="n">
+        <v>0</v>
+      </c>
+      <c r="U74" t="n">
+        <v>0</v>
+      </c>
+      <c r="V74" t="n">
+        <v>0</v>
+      </c>
+      <c r="W74" t="n">
+        <v>0</v>
+      </c>
+      <c r="X74" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y74" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z74" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>527</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ZSN - Náhrada PN</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M75" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" t="n">
+        <v>197.6</v>
+      </c>
+      <c r="P75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>197.6</v>
+      </c>
+      <c r="R75" t="n">
+        <v>0</v>
+      </c>
+      <c r="S75" t="n">
+        <v>197.6</v>
+      </c>
+      <c r="T75" t="n">
+        <v>0</v>
+      </c>
+      <c r="U75" t="n">
+        <v>0</v>
+      </c>
+      <c r="V75" t="n">
+        <v>0</v>
+      </c>
+      <c r="W75" t="n">
+        <v>0</v>
+      </c>
+      <c r="X75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y75" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z75" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>528</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Stravovanie nad limit</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M76" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="n">
+        <v>122.9</v>
+      </c>
+      <c r="P76" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>122.9</v>
+      </c>
+      <c r="R76" t="n">
+        <v>0</v>
+      </c>
+      <c r="S76" t="n">
+        <v>122.9</v>
+      </c>
+      <c r="T76" t="n">
+        <v>0</v>
+      </c>
+      <c r="U76" t="n">
+        <v>0</v>
+      </c>
+      <c r="V76" t="n">
+        <v>0</v>
+      </c>
+      <c r="W76" t="n">
+        <v>0</v>
+      </c>
+      <c r="X76" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y76" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z76" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>538</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Transakčná daň</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M77" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" t="n">
+        <v>80.07</v>
+      </c>
+      <c r="P77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>80.07</v>
+      </c>
+      <c r="R77" t="n">
+        <v>0</v>
+      </c>
+      <c r="S77" t="n">
+        <v>80.07</v>
+      </c>
+      <c r="T77" t="n">
+        <v>0</v>
+      </c>
+      <c r="U77" t="n">
+        <v>0</v>
+      </c>
+      <c r="V77" t="n">
+        <v>0</v>
+      </c>
+      <c r="W77" t="n">
+        <v>0</v>
+      </c>
+      <c r="X77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y77" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z77" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>548</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Poistenie</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M78" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" t="n">
+        <v>194.83</v>
+      </c>
+      <c r="P78" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>194.83</v>
+      </c>
+      <c r="R78" t="n">
+        <v>0</v>
+      </c>
+      <c r="S78" t="n">
+        <v>194.83</v>
+      </c>
+      <c r="T78" t="n">
+        <v>0</v>
+      </c>
+      <c r="U78" t="n">
+        <v>0</v>
+      </c>
+      <c r="V78" t="n">
+        <v>0</v>
+      </c>
+      <c r="W78" t="n">
+        <v>0</v>
+      </c>
+      <c r="X78" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y78" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z78" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>551</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Odpisy osobné automobily</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" t="n">
+        <v>962.89</v>
+      </c>
+      <c r="P79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>962.89</v>
+      </c>
+      <c r="R79" t="n">
+        <v>0</v>
+      </c>
+      <c r="S79" t="n">
+        <v>962.89</v>
+      </c>
+      <c r="T79" t="n">
+        <v>0</v>
+      </c>
+      <c r="U79" t="n">
+        <v>0</v>
+      </c>
+      <c r="V79" t="n">
+        <v>0</v>
+      </c>
+      <c r="W79" t="n">
+        <v>0</v>
+      </c>
+      <c r="X79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y79" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z79" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>551</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Odpisy stroje,prístroje</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" t="n">
+        <v>176.28</v>
+      </c>
+      <c r="P80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>176.28</v>
+      </c>
+      <c r="R80" t="n">
+        <v>0</v>
+      </c>
+      <c r="S80" t="n">
+        <v>176.28</v>
+      </c>
+      <c r="T80" t="n">
+        <v>0</v>
+      </c>
+      <c r="U80" t="n">
+        <v>0</v>
+      </c>
+      <c r="V80" t="n">
+        <v>0</v>
+      </c>
+      <c r="W80" t="n">
+        <v>0</v>
+      </c>
+      <c r="X80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z80" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>562</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Nákladové úroky AA944RK</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>153.51</v>
+      </c>
+      <c r="P81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>153.51</v>
+      </c>
+      <c r="R81" t="n">
+        <v>0</v>
+      </c>
+      <c r="S81" t="n">
+        <v>153.51</v>
+      </c>
+      <c r="T81" t="n">
+        <v>0</v>
+      </c>
+      <c r="U81" t="n">
+        <v>0</v>
+      </c>
+      <c r="V81" t="n">
+        <v>0</v>
+      </c>
+      <c r="W81" t="n">
+        <v>0</v>
+      </c>
+      <c r="X81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y81" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z81" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>562</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Nákladové úroky</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M82" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0</v>
+      </c>
+      <c r="O82" t="n">
+        <v>108.1</v>
+      </c>
+      <c r="P82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>108.1</v>
+      </c>
+      <c r="R82" t="n">
+        <v>0</v>
+      </c>
+      <c r="S82" t="n">
+        <v>108.1</v>
+      </c>
+      <c r="T82" t="n">
+        <v>0</v>
+      </c>
+      <c r="U82" t="n">
+        <v>0</v>
+      </c>
+      <c r="V82" t="n">
+        <v>0</v>
+      </c>
+      <c r="W82" t="n">
+        <v>0</v>
+      </c>
+      <c r="X82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y82" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z82" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>568</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Bankové poplatky</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N83" t="n">
+        <v>0</v>
+      </c>
+      <c r="O83" t="n">
+        <v>31.61</v>
+      </c>
+      <c r="P83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>31.61</v>
+      </c>
+      <c r="R83" t="n">
+        <v>0</v>
+      </c>
+      <c r="S83" t="n">
+        <v>31.61</v>
+      </c>
+      <c r="T83" t="n">
+        <v>0</v>
+      </c>
+      <c r="U83" t="n">
+        <v>0</v>
+      </c>
+      <c r="V83" t="n">
+        <v>0</v>
+      </c>
+      <c r="W83" t="n">
+        <v>0</v>
+      </c>
+      <c r="X83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y83" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z83" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t>601</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>040</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>AMADYS -Tržby za vlastné výrobky</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="M66" t="n">
-        <v>0</v>
-      </c>
-      <c r="N66" t="n">
-        <v>0</v>
-      </c>
-      <c r="O66" t="n">
-        <v>0</v>
-      </c>
-      <c r="P66" t="n">
+      <c r="M84" t="n">
+        <v>0</v>
+      </c>
+      <c r="N84" t="n">
+        <v>0</v>
+      </c>
+      <c r="O84" t="n">
+        <v>0</v>
+      </c>
+      <c r="P84" t="n">
         <v>78867.97</v>
       </c>
-      <c r="Q66" t="n">
-        <v>0</v>
-      </c>
-      <c r="R66" t="n">
+      <c r="Q84" t="n">
+        <v>0</v>
+      </c>
+      <c r="R84" t="n">
         <v>78867.97</v>
       </c>
-      <c r="S66" t="n">
+      <c r="S84" t="n">
         <v>-78867.97</v>
       </c>
-      <c r="T66" t="n">
-        <v>0</v>
-      </c>
-      <c r="U66" t="n">
-        <v>0</v>
-      </c>
-      <c r="V66" t="n">
-        <v>0</v>
-      </c>
-      <c r="W66" t="n">
-        <v>0</v>
-      </c>
-      <c r="X66" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y66" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z66" t="n">
+      <c r="T84" t="n">
+        <v>0</v>
+      </c>
+      <c r="U84" t="n">
+        <v>0</v>
+      </c>
+      <c r="V84" t="n">
+        <v>0</v>
+      </c>
+      <c r="W84" t="n">
+        <v>0</v>
+      </c>
+      <c r="X84" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y84" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z84" t="n">
         <v>2026</v>
       </c>
     </row>

</xml_diff>